<commit_message>
Add new contractor management features and update templates
- Updated index.html to include a dropdown for selecting contractors and added fields for new contractor registration.
- Enhanced script.js to load contractors and handle new contractor registration.
- Introduced new JSON configuration for contractors and updated routes to fetch contractor data.
- Added new utility for managing contractors in contrataadasConfig.js.
- Updated styles.css for improved layout and spacing.
- Added new templates for KORAES and updated existing templates.
</commit_message>
<xml_diff>
--- a/templates/template_HACDF.xlsx
+++ b/templates/template_HACDF.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD966DE6-03D9-4588-AD67-30782A4B7F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF6D853F-F5D8-45A5-9DE1-F5F4B4AF59D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -235,13 +235,13 @@
     <t>BOLETIM DE MEDIÇÃO DE SERVIÇOS (BMS)</t>
   </si>
   <si>
-    <t>Nº Pedido de Compra</t>
+    <t>Nº Pedido de Compra:</t>
   </si>
   <si>
     <t>Objeto:</t>
   </si>
   <si>
-    <t>Vencimento NF:</t>
+    <t>Vencimento:</t>
   </si>
   <si>
     <t>Data de Início (OS):</t>
@@ -385,7 +385,7 @@
     <t>CC</t>
   </si>
   <si>
-    <t xml:space="preserve">Gerente do Projeto: </t>
+    <t xml:space="preserve">Documentação Conferida: </t>
   </si>
   <si>
     <t>CONCLUÍDO</t>
@@ -1227,13 +1227,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="139">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1249,7 +1249,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1331,7 +1331,7 @@
     <xf numFmtId="167" fontId="8" fillId="3" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="167" fontId="9" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1365,7 +1365,7 @@
     <xf numFmtId="166" fontId="6" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="9" fillId="4" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1399,29 +1399,25 @@
     <xf numFmtId="167" fontId="6" fillId="5" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1431,47 +1427,33 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="7" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1481,16 +1463,12 @@
     <xf numFmtId="14" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1503,8 +1481,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1514,19 +1490,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1548,14 +1520,12 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="6" fillId="5" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1571,6 +1541,34 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1593,22 +1591,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>638175</xdr:colOff>
+      <xdr:colOff>704850</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>-9525</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>619125</xdr:colOff>
+      <xdr:colOff>571500</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Imagem 5">
+        <xdr:cNvPr id="12" name="Imagem 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D752A8B-729A-39E5-9823-79413EC9E3C3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64C3FB5E-4757-A16F-11E8-2A32C7BA3239}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1624,8 +1622,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12934950" y="-9525"/>
-          <a:ext cx="2057400" cy="1152525"/>
+          <a:off x="13001625" y="0"/>
+          <a:ext cx="1943100" cy="1085850"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1894,32 +1892,30 @@
     </row>
     <row r="2" spans="1:26" ht="24.75" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="123"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="106"/>
-      <c r="E2" s="125" t="s">
+      <c r="B2" s="96"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="97" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="106"/>
-      <c r="J2" s="125" t="s">
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="112"/>
+      <c r="J2" s="97" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="91"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="106"/>
-      <c r="O2" s="123"/>
-      <c r="P2" s="91"/>
-      <c r="Q2" s="106"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="96"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="112"/>
       <c r="R2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S2" s="5">
-        <v>1</v>
-      </c>
+      <c r="S2" s="5"/>
       <c r="T2" s="66" t="s">
         <v>3</v>
       </c>
@@ -1932,28 +1928,28 @@
     </row>
     <row r="3" spans="1:26" ht="44.25" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="124"/>
-      <c r="C3" s="113"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="128"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="113"/>
-      <c r="L3" s="113"/>
-      <c r="M3" s="113"/>
-      <c r="N3" s="114"/>
-      <c r="O3" s="124"/>
-      <c r="P3" s="113"/>
-      <c r="Q3" s="114"/>
-      <c r="R3" s="109" t="s">
+      <c r="B3" s="113"/>
+      <c r="C3" s="114"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="99"/>
+      <c r="G3" s="99"/>
+      <c r="H3" s="99"/>
+      <c r="I3" s="100"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="114"/>
+      <c r="L3" s="114"/>
+      <c r="M3" s="114"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="113"/>
+      <c r="P3" s="114"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="S3" s="73"/>
-      <c r="T3" s="110"/>
-      <c r="U3" s="103"/>
+      <c r="S3" s="116"/>
+      <c r="T3" s="88"/>
+      <c r="U3" s="117"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
@@ -1962,30 +1958,30 @@
     </row>
     <row r="4" spans="1:26" ht="27.75" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="115" t="s">
+      <c r="B4" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="94"/>
-      <c r="D4" s="94"/>
-      <c r="E4" s="94"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="94"/>
-      <c r="J4" s="94"/>
-      <c r="K4" s="94"/>
-      <c r="L4" s="94"/>
-      <c r="M4" s="94"/>
-      <c r="N4" s="94"/>
-      <c r="O4" s="94"/>
-      <c r="P4" s="94"/>
-      <c r="Q4" s="94"/>
-      <c r="R4" s="109" t="s">
+      <c r="C4" s="118"/>
+      <c r="D4" s="118"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="118"/>
+      <c r="G4" s="118"/>
+      <c r="H4" s="118"/>
+      <c r="I4" s="118"/>
+      <c r="J4" s="118"/>
+      <c r="K4" s="118"/>
+      <c r="L4" s="118"/>
+      <c r="M4" s="118"/>
+      <c r="N4" s="118"/>
+      <c r="O4" s="118"/>
+      <c r="P4" s="118"/>
+      <c r="Q4" s="118"/>
+      <c r="R4" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="S4" s="73"/>
-      <c r="T4" s="116"/>
-      <c r="U4" s="103"/>
+      <c r="S4" s="116"/>
+      <c r="T4" s="92"/>
+      <c r="U4" s="117"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
@@ -1994,30 +1990,30 @@
     </row>
     <row r="5" spans="1:26" ht="27.75" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="117" t="s">
+      <c r="B5" s="93" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="82"/>
-      <c r="D5" s="119"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81"/>
-      <c r="L5" s="81"/>
-      <c r="M5" s="81"/>
-      <c r="N5" s="81"/>
-      <c r="O5" s="81"/>
-      <c r="P5" s="81"/>
-      <c r="Q5" s="120"/>
-      <c r="R5" s="122" t="s">
+      <c r="C5" s="119"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="120"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="120"/>
+      <c r="H5" s="120"/>
+      <c r="I5" s="120"/>
+      <c r="J5" s="120"/>
+      <c r="K5" s="120"/>
+      <c r="L5" s="120"/>
+      <c r="M5" s="120"/>
+      <c r="N5" s="120"/>
+      <c r="O5" s="120"/>
+      <c r="P5" s="120"/>
+      <c r="Q5" s="121"/>
+      <c r="R5" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="S5" s="73"/>
-      <c r="T5" s="111"/>
-      <c r="U5" s="103"/>
+      <c r="S5" s="116"/>
+      <c r="T5" s="89"/>
+      <c r="U5" s="117"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
@@ -2026,28 +2022,28 @@
     </row>
     <row r="6" spans="1:26" ht="27.75" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="118"/>
-      <c r="C6" s="95"/>
-      <c r="D6" s="93"/>
-      <c r="E6" s="94"/>
-      <c r="F6" s="94"/>
-      <c r="G6" s="94"/>
-      <c r="H6" s="94"/>
-      <c r="I6" s="94"/>
-      <c r="J6" s="94"/>
-      <c r="K6" s="94"/>
-      <c r="L6" s="94"/>
-      <c r="M6" s="94"/>
-      <c r="N6" s="94"/>
-      <c r="O6" s="94"/>
-      <c r="P6" s="94"/>
-      <c r="Q6" s="121"/>
+      <c r="B6" s="122"/>
+      <c r="C6" s="123"/>
+      <c r="D6" s="124"/>
+      <c r="E6" s="118"/>
+      <c r="F6" s="118"/>
+      <c r="G6" s="118"/>
+      <c r="H6" s="118"/>
+      <c r="I6" s="118"/>
+      <c r="J6" s="118"/>
+      <c r="K6" s="118"/>
+      <c r="L6" s="118"/>
+      <c r="M6" s="118"/>
+      <c r="N6" s="118"/>
+      <c r="O6" s="118"/>
+      <c r="P6" s="118"/>
+      <c r="Q6" s="125"/>
       <c r="R6" s="7" t="s">
         <v>9</v>
       </c>
       <c r="S6" s="8"/>
-      <c r="T6" s="102"/>
-      <c r="U6" s="103"/>
+      <c r="T6" s="84"/>
+      <c r="U6" s="117"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
@@ -2056,30 +2052,30 @@
     </row>
     <row r="7" spans="1:26" ht="27.75" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="80" t="s">
+      <c r="B7" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="81"/>
-      <c r="D7" s="82"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="81"/>
-      <c r="G7" s="81"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="81"/>
-      <c r="K7" s="81"/>
-      <c r="L7" s="81"/>
-      <c r="M7" s="81"/>
-      <c r="N7" s="81"/>
-      <c r="O7" s="81"/>
-      <c r="P7" s="81"/>
-      <c r="Q7" s="81"/>
-      <c r="R7" s="84" t="s">
+      <c r="C7" s="120"/>
+      <c r="D7" s="119"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="120"/>
+      <c r="H7" s="120"/>
+      <c r="I7" s="120"/>
+      <c r="J7" s="120"/>
+      <c r="K7" s="120"/>
+      <c r="L7" s="120"/>
+      <c r="M7" s="120"/>
+      <c r="N7" s="120"/>
+      <c r="O7" s="120"/>
+      <c r="P7" s="120"/>
+      <c r="Q7" s="120"/>
+      <c r="R7" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="S7" s="85"/>
-      <c r="T7" s="102"/>
-      <c r="U7" s="103"/>
+      <c r="S7" s="126"/>
+      <c r="T7" s="84"/>
+      <c r="U7" s="117"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
@@ -2088,44 +2084,44 @@
     </row>
     <row r="8" spans="1:26" ht="24" customHeight="1">
       <c r="A8" s="9"/>
-      <c r="B8" s="86" t="s">
+      <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="88" t="s">
+      <c r="C8" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="90" t="s">
+      <c r="D8" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="91"/>
-      <c r="F8" s="92"/>
-      <c r="G8" s="90" t="s">
+      <c r="E8" s="111"/>
+      <c r="F8" s="127"/>
+      <c r="G8" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="97" t="s">
+      <c r="H8" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="98"/>
-      <c r="J8" s="99"/>
-      <c r="K8" s="100" t="s">
+      <c r="I8" s="128"/>
+      <c r="J8" s="129"/>
+      <c r="K8" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="L8" s="98"/>
-      <c r="M8" s="98"/>
-      <c r="N8" s="99"/>
-      <c r="O8" s="101" t="s">
+      <c r="L8" s="128"/>
+      <c r="M8" s="128"/>
+      <c r="N8" s="129"/>
+      <c r="O8" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="P8" s="98"/>
-      <c r="Q8" s="98"/>
-      <c r="R8" s="99"/>
-      <c r="S8" s="96" t="s">
+      <c r="P8" s="128"/>
+      <c r="Q8" s="128"/>
+      <c r="R8" s="129"/>
+      <c r="S8" s="80" t="s">
         <v>19</v>
       </c>
-      <c r="T8" s="104" t="s">
+      <c r="T8" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="U8" s="99"/>
+      <c r="U8" s="129"/>
       <c r="V8" s="9"/>
       <c r="W8" s="9"/>
       <c r="X8" s="9"/>
@@ -2134,12 +2130,12 @@
     </row>
     <row r="9" spans="1:26" ht="24" customHeight="1">
       <c r="A9" s="9"/>
-      <c r="B9" s="87"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="94"/>
-      <c r="F9" s="95"/>
-      <c r="G9" s="93"/>
+      <c r="B9" s="130"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="124"/>
+      <c r="E9" s="118"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="124"/>
       <c r="H9" s="10" t="s">
         <v>21</v>
       </c>
@@ -2173,7 +2169,7 @@
       <c r="R9" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="S9" s="87"/>
+      <c r="S9" s="130"/>
       <c r="T9" s="19" t="s">
         <v>21</v>
       </c>
@@ -2186,15 +2182,15 @@
       <c r="Y9" s="9"/>
       <c r="Z9" s="9"/>
     </row>
-    <row r="10" spans="1:26" ht="53.25" customHeight="1">
+    <row r="10" spans="1:26" ht="39.75" customHeight="1">
       <c r="A10" s="21"/>
       <c r="B10" s="22" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="22"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="72"/>
-      <c r="F10" s="73"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="132"/>
+      <c r="F10" s="116"/>
       <c r="G10" s="34"/>
       <c r="H10" s="23"/>
       <c r="I10" s="33"/>
@@ -2222,9 +2218,9 @@
         <v>29</v>
       </c>
       <c r="C11" s="22"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="74"/>
-      <c r="F11" s="75"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="71"/>
       <c r="G11" s="34"/>
       <c r="H11" s="23"/>
       <c r="I11" s="33"/>
@@ -2252,9 +2248,9 @@
         <v>30</v>
       </c>
       <c r="C12" s="22"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="72"/>
-      <c r="F12" s="73"/>
+      <c r="D12" s="69"/>
+      <c r="E12" s="132"/>
+      <c r="F12" s="116"/>
       <c r="G12" s="34"/>
       <c r="H12" s="23"/>
       <c r="I12" s="33"/>
@@ -2276,15 +2272,15 @@
       <c r="Y12" s="21"/>
       <c r="Z12" s="21"/>
     </row>
-    <row r="13" spans="1:26" s="68" customFormat="1" ht="60" customHeight="1">
+    <row r="13" spans="1:26" ht="60" customHeight="1">
       <c r="A13" s="21"/>
       <c r="B13" s="22" t="s">
         <v>31</v>
       </c>
       <c r="C13" s="22"/>
-      <c r="D13" s="71"/>
-      <c r="E13" s="72"/>
-      <c r="F13" s="73"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="132"/>
+      <c r="F13" s="116"/>
       <c r="G13" s="34"/>
       <c r="H13" s="23"/>
       <c r="I13" s="33"/>
@@ -2306,15 +2302,15 @@
       <c r="Y13" s="21"/>
       <c r="Z13" s="21"/>
     </row>
-    <row r="14" spans="1:26" s="68" customFormat="1" ht="60" customHeight="1">
+    <row r="14" spans="1:26" ht="60" customHeight="1">
       <c r="A14" s="21"/>
       <c r="B14" s="22" t="s">
         <v>32</v>
       </c>
       <c r="C14" s="22"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="72"/>
-      <c r="F14" s="73"/>
+      <c r="D14" s="69"/>
+      <c r="E14" s="132"/>
+      <c r="F14" s="116"/>
       <c r="G14" s="34"/>
       <c r="H14" s="23"/>
       <c r="I14" s="33"/>
@@ -2336,15 +2332,15 @@
       <c r="Y14" s="21"/>
       <c r="Z14" s="21"/>
     </row>
-    <row r="15" spans="1:26" s="68" customFormat="1" ht="60" customHeight="1">
+    <row r="15" spans="1:26" ht="60" customHeight="1">
       <c r="A15" s="21"/>
       <c r="B15" s="22" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="22"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="72"/>
-      <c r="F15" s="73"/>
+      <c r="D15" s="69"/>
+      <c r="E15" s="132"/>
+      <c r="F15" s="116"/>
       <c r="G15" s="34"/>
       <c r="H15" s="23"/>
       <c r="I15" s="33"/>
@@ -2366,15 +2362,15 @@
       <c r="Y15" s="21"/>
       <c r="Z15" s="21"/>
     </row>
-    <row r="16" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="16" spans="1:26" ht="60" customHeight="1">
       <c r="A16" s="21"/>
       <c r="B16" s="22" t="s">
         <v>34</v>
       </c>
       <c r="C16" s="22"/>
-      <c r="D16" s="71"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="73"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="132"/>
+      <c r="F16" s="116"/>
       <c r="G16" s="34"/>
       <c r="H16" s="23"/>
       <c r="I16" s="33"/>
@@ -2396,15 +2392,15 @@
       <c r="Y16" s="21"/>
       <c r="Z16" s="21"/>
     </row>
-    <row r="17" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="17" spans="1:26" ht="60" customHeight="1">
       <c r="A17" s="21"/>
       <c r="B17" s="22" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="22"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="72"/>
-      <c r="F17" s="73"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="132"/>
+      <c r="F17" s="116"/>
       <c r="G17" s="34"/>
       <c r="H17" s="23"/>
       <c r="I17" s="33"/>
@@ -2426,15 +2422,15 @@
       <c r="Y17" s="21"/>
       <c r="Z17" s="21"/>
     </row>
-    <row r="18" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="18" spans="1:26" ht="60" customHeight="1">
       <c r="A18" s="21"/>
       <c r="B18" s="22" t="s">
         <v>36</v>
       </c>
       <c r="C18" s="22"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="72"/>
-      <c r="F18" s="73"/>
+      <c r="D18" s="69"/>
+      <c r="E18" s="132"/>
+      <c r="F18" s="116"/>
       <c r="G18" s="34"/>
       <c r="H18" s="23"/>
       <c r="I18" s="33"/>
@@ -2456,15 +2452,15 @@
       <c r="Y18" s="21"/>
       <c r="Z18" s="21"/>
     </row>
-    <row r="19" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="19" spans="1:26" ht="60" customHeight="1">
       <c r="A19" s="21"/>
       <c r="B19" s="22" t="s">
         <v>37</v>
       </c>
       <c r="C19" s="22"/>
-      <c r="D19" s="71"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="73"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="132"/>
+      <c r="F19" s="116"/>
       <c r="G19" s="34"/>
       <c r="H19" s="23"/>
       <c r="I19" s="33"/>
@@ -2486,15 +2482,15 @@
       <c r="Y19" s="21"/>
       <c r="Z19" s="21"/>
     </row>
-    <row r="20" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="20" spans="1:26" ht="60" customHeight="1">
       <c r="A20" s="21"/>
       <c r="B20" s="22" t="s">
         <v>38</v>
       </c>
       <c r="C20" s="22"/>
-      <c r="D20" s="71"/>
-      <c r="E20" s="72"/>
-      <c r="F20" s="73"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="132"/>
+      <c r="F20" s="116"/>
       <c r="G20" s="34"/>
       <c r="H20" s="23"/>
       <c r="I20" s="33"/>
@@ -2516,15 +2512,15 @@
       <c r="Y20" s="21"/>
       <c r="Z20" s="21"/>
     </row>
-    <row r="21" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="21" spans="1:26" ht="60" customHeight="1">
       <c r="A21" s="21"/>
       <c r="B21" s="22" t="s">
         <v>39</v>
       </c>
       <c r="C21" s="22"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="72"/>
-      <c r="F21" s="73"/>
+      <c r="D21" s="69"/>
+      <c r="E21" s="132"/>
+      <c r="F21" s="116"/>
       <c r="G21" s="34"/>
       <c r="H21" s="23"/>
       <c r="I21" s="33"/>
@@ -2546,15 +2542,15 @@
       <c r="Y21" s="21"/>
       <c r="Z21" s="21"/>
     </row>
-    <row r="22" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="22" spans="1:26" ht="60" customHeight="1">
       <c r="A22" s="21"/>
       <c r="B22" s="22" t="s">
         <v>40</v>
       </c>
       <c r="C22" s="22"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="72"/>
-      <c r="F22" s="73"/>
+      <c r="D22" s="69"/>
+      <c r="E22" s="132"/>
+      <c r="F22" s="116"/>
       <c r="G22" s="34"/>
       <c r="H22" s="23"/>
       <c r="I22" s="33"/>
@@ -2576,15 +2572,15 @@
       <c r="Y22" s="21"/>
       <c r="Z22" s="21"/>
     </row>
-    <row r="23" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="23" spans="1:26" ht="60" customHeight="1">
       <c r="A23" s="21"/>
       <c r="B23" s="22" t="s">
         <v>41</v>
       </c>
       <c r="C23" s="22"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="72"/>
-      <c r="F23" s="73"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="132"/>
+      <c r="F23" s="116"/>
       <c r="G23" s="34"/>
       <c r="H23" s="23"/>
       <c r="I23" s="33"/>
@@ -2606,15 +2602,15 @@
       <c r="Y23" s="21"/>
       <c r="Z23" s="21"/>
     </row>
-    <row r="24" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="24" spans="1:26" ht="60" customHeight="1">
       <c r="A24" s="21"/>
       <c r="B24" s="22" t="s">
         <v>42</v>
       </c>
       <c r="C24" s="22"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="72"/>
-      <c r="F24" s="73"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="132"/>
+      <c r="F24" s="116"/>
       <c r="G24" s="34"/>
       <c r="H24" s="23"/>
       <c r="I24" s="33"/>
@@ -2636,15 +2632,15 @@
       <c r="Y24" s="21"/>
       <c r="Z24" s="21"/>
     </row>
-    <row r="25" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="25" spans="1:26" ht="60" customHeight="1">
       <c r="A25" s="21"/>
       <c r="B25" s="22" t="s">
         <v>43</v>
       </c>
       <c r="C25" s="22"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="72"/>
-      <c r="F25" s="73"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="132"/>
+      <c r="F25" s="116"/>
       <c r="G25" s="34"/>
       <c r="H25" s="23"/>
       <c r="I25" s="33"/>
@@ -2666,15 +2662,15 @@
       <c r="Y25" s="21"/>
       <c r="Z25" s="21"/>
     </row>
-    <row r="26" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="26" spans="1:26" ht="60" customHeight="1">
       <c r="A26" s="21"/>
       <c r="B26" s="22" t="s">
         <v>44</v>
       </c>
       <c r="C26" s="22"/>
-      <c r="D26" s="71"/>
-      <c r="E26" s="72"/>
-      <c r="F26" s="73"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="132"/>
+      <c r="F26" s="116"/>
       <c r="G26" s="34"/>
       <c r="H26" s="23"/>
       <c r="I26" s="33"/>
@@ -2696,15 +2692,15 @@
       <c r="Y26" s="21"/>
       <c r="Z26" s="21"/>
     </row>
-    <row r="27" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="27" spans="1:26" ht="60" customHeight="1">
       <c r="A27" s="21"/>
       <c r="B27" s="22" t="s">
         <v>45</v>
       </c>
       <c r="C27" s="22"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="72"/>
-      <c r="F27" s="73"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="132"/>
+      <c r="F27" s="116"/>
       <c r="G27" s="34"/>
       <c r="H27" s="23"/>
       <c r="I27" s="33"/>
@@ -2726,15 +2722,15 @@
       <c r="Y27" s="21"/>
       <c r="Z27" s="21"/>
     </row>
-    <row r="28" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="28" spans="1:26" ht="60" customHeight="1">
       <c r="A28" s="21"/>
       <c r="B28" s="22" t="s">
         <v>46</v>
       </c>
       <c r="C28" s="22"/>
-      <c r="D28" s="71"/>
-      <c r="E28" s="72"/>
-      <c r="F28" s="73"/>
+      <c r="D28" s="69"/>
+      <c r="E28" s="132"/>
+      <c r="F28" s="116"/>
       <c r="G28" s="34"/>
       <c r="H28" s="23"/>
       <c r="I28" s="33"/>
@@ -2756,15 +2752,15 @@
       <c r="Y28" s="21"/>
       <c r="Z28" s="21"/>
     </row>
-    <row r="29" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="29" spans="1:26" ht="60" customHeight="1">
       <c r="A29" s="21"/>
       <c r="B29" s="22" t="s">
         <v>47</v>
       </c>
       <c r="C29" s="22"/>
-      <c r="D29" s="71"/>
-      <c r="E29" s="72"/>
-      <c r="F29" s="73"/>
+      <c r="D29" s="69"/>
+      <c r="E29" s="132"/>
+      <c r="F29" s="116"/>
       <c r="G29" s="34"/>
       <c r="H29" s="23"/>
       <c r="I29" s="33"/>
@@ -2786,15 +2782,15 @@
       <c r="Y29" s="21"/>
       <c r="Z29" s="21"/>
     </row>
-    <row r="30" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="30" spans="1:26" ht="60" customHeight="1">
       <c r="A30" s="21"/>
       <c r="B30" s="22" t="s">
         <v>48</v>
       </c>
       <c r="C30" s="22"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="72"/>
-      <c r="F30" s="73"/>
+      <c r="D30" s="69"/>
+      <c r="E30" s="132"/>
+      <c r="F30" s="116"/>
       <c r="G30" s="34"/>
       <c r="H30" s="23"/>
       <c r="I30" s="33"/>
@@ -2816,15 +2812,15 @@
       <c r="Y30" s="21"/>
       <c r="Z30" s="21"/>
     </row>
-    <row r="31" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="31" spans="1:26" ht="60" customHeight="1">
       <c r="A31" s="21"/>
       <c r="B31" s="22" t="s">
         <v>49</v>
       </c>
       <c r="C31" s="22"/>
-      <c r="D31" s="71"/>
-      <c r="E31" s="72"/>
-      <c r="F31" s="73"/>
+      <c r="D31" s="69"/>
+      <c r="E31" s="132"/>
+      <c r="F31" s="116"/>
       <c r="G31" s="34"/>
       <c r="H31" s="23"/>
       <c r="I31" s="33"/>
@@ -2846,15 +2842,15 @@
       <c r="Y31" s="21"/>
       <c r="Z31" s="21"/>
     </row>
-    <row r="32" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="32" spans="1:26" ht="60" customHeight="1">
       <c r="A32" s="21"/>
       <c r="B32" s="22" t="s">
         <v>50</v>
       </c>
       <c r="C32" s="22"/>
-      <c r="D32" s="71"/>
-      <c r="E32" s="72"/>
-      <c r="F32" s="73"/>
+      <c r="D32" s="69"/>
+      <c r="E32" s="132"/>
+      <c r="F32" s="116"/>
       <c r="G32" s="34"/>
       <c r="H32" s="23"/>
       <c r="I32" s="33"/>
@@ -2876,15 +2872,15 @@
       <c r="Y32" s="21"/>
       <c r="Z32" s="21"/>
     </row>
-    <row r="33" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="33" spans="1:26" ht="60" customHeight="1">
       <c r="A33" s="21"/>
       <c r="B33" s="22" t="s">
         <v>51</v>
       </c>
       <c r="C33" s="22"/>
-      <c r="D33" s="71"/>
-      <c r="E33" s="72"/>
-      <c r="F33" s="73"/>
+      <c r="D33" s="69"/>
+      <c r="E33" s="132"/>
+      <c r="F33" s="116"/>
       <c r="G33" s="34"/>
       <c r="H33" s="23"/>
       <c r="I33" s="33"/>
@@ -2906,15 +2902,15 @@
       <c r="Y33" s="21"/>
       <c r="Z33" s="21"/>
     </row>
-    <row r="34" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="34" spans="1:26" ht="60" customHeight="1">
       <c r="A34" s="21"/>
       <c r="B34" s="22" t="s">
         <v>52</v>
       </c>
       <c r="C34" s="22"/>
-      <c r="D34" s="71"/>
-      <c r="E34" s="72"/>
-      <c r="F34" s="73"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="132"/>
+      <c r="F34" s="116"/>
       <c r="G34" s="34"/>
       <c r="H34" s="23"/>
       <c r="I34" s="33"/>
@@ -2936,15 +2932,15 @@
       <c r="Y34" s="21"/>
       <c r="Z34" s="21"/>
     </row>
-    <row r="35" spans="1:26" s="69" customFormat="1" ht="60" customHeight="1">
+    <row r="35" spans="1:26" ht="60" customHeight="1">
       <c r="A35" s="21"/>
       <c r="B35" s="22" t="s">
         <v>53</v>
       </c>
       <c r="C35" s="22"/>
-      <c r="D35" s="71"/>
-      <c r="E35" s="72"/>
-      <c r="F35" s="73"/>
+      <c r="D35" s="69"/>
+      <c r="E35" s="132"/>
+      <c r="F35" s="116"/>
       <c r="G35" s="34"/>
       <c r="H35" s="23"/>
       <c r="I35" s="33"/>
@@ -2968,14 +2964,14 @@
     </row>
     <row r="36" spans="1:26" ht="33" customHeight="1">
       <c r="A36" s="37"/>
-      <c r="B36" s="76"/>
-      <c r="C36" s="77"/>
-      <c r="D36" s="78" t="s">
+      <c r="B36" s="72"/>
+      <c r="C36" s="133"/>
+      <c r="D36" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="E36" s="79"/>
-      <c r="F36" s="77"/>
-      <c r="G36" s="70"/>
+      <c r="E36" s="134"/>
+      <c r="F36" s="133"/>
+      <c r="G36" s="68"/>
       <c r="H36" s="38"/>
       <c r="I36" s="39"/>
       <c r="J36" s="40">
@@ -3019,15 +3015,15 @@
     </row>
     <row r="37" spans="1:26" ht="19.5" customHeight="1">
       <c r="A37" s="37"/>
-      <c r="B37" s="131"/>
-      <c r="C37" s="91"/>
-      <c r="D37" s="91"/>
-      <c r="E37" s="91"/>
-      <c r="F37" s="91"/>
-      <c r="G37" s="91"/>
-      <c r="H37" s="91"/>
-      <c r="I37" s="91"/>
-      <c r="J37" s="91"/>
+      <c r="B37" s="103"/>
+      <c r="C37" s="111"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="111"/>
+      <c r="H37" s="111"/>
+      <c r="I37" s="111"/>
+      <c r="J37" s="111"/>
       <c r="K37" s="50" t="s">
         <v>55</v>
       </c>
@@ -3037,13 +3033,13 @@
         <f t="shared" ref="N37:N38" si="0">SUMIF($G$10,M37,$N$10)</f>
         <v>0</v>
       </c>
-      <c r="O37" s="105"/>
-      <c r="P37" s="91"/>
-      <c r="Q37" s="91"/>
-      <c r="R37" s="91"/>
-      <c r="S37" s="91"/>
-      <c r="T37" s="91"/>
-      <c r="U37" s="106"/>
+      <c r="O37" s="86"/>
+      <c r="P37" s="111"/>
+      <c r="Q37" s="111"/>
+      <c r="R37" s="111"/>
+      <c r="S37" s="111"/>
+      <c r="T37" s="111"/>
+      <c r="U37" s="112"/>
       <c r="V37" s="49"/>
       <c r="W37" s="37"/>
       <c r="X37" s="37"/>
@@ -3052,15 +3048,15 @@
     </row>
     <row r="38" spans="1:26" ht="19.5" customHeight="1">
       <c r="A38" s="37"/>
-      <c r="B38" s="132"/>
-      <c r="C38" s="107"/>
-      <c r="D38" s="107"/>
-      <c r="E38" s="107"/>
-      <c r="F38" s="107"/>
-      <c r="G38" s="107"/>
-      <c r="H38" s="107"/>
-      <c r="I38" s="107"/>
-      <c r="J38" s="107"/>
+      <c r="B38" s="135"/>
+      <c r="C38" s="136"/>
+      <c r="D38" s="136"/>
+      <c r="E38" s="136"/>
+      <c r="F38" s="136"/>
+      <c r="G38" s="136"/>
+      <c r="H38" s="136"/>
+      <c r="I38" s="136"/>
+      <c r="J38" s="136"/>
       <c r="K38" s="54"/>
       <c r="L38" s="55"/>
       <c r="M38" s="55"/>
@@ -3068,13 +3064,13 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O38" s="107"/>
-      <c r="P38" s="107"/>
-      <c r="Q38" s="107"/>
-      <c r="R38" s="107"/>
-      <c r="S38" s="107"/>
-      <c r="T38" s="107"/>
-      <c r="U38" s="108"/>
+      <c r="O38" s="136"/>
+      <c r="P38" s="136"/>
+      <c r="Q38" s="136"/>
+      <c r="R38" s="136"/>
+      <c r="S38" s="136"/>
+      <c r="T38" s="136"/>
+      <c r="U38" s="137"/>
       <c r="V38" s="49"/>
       <c r="W38" s="37"/>
       <c r="X38" s="37"/>
@@ -3083,13 +3079,13 @@
     </row>
     <row r="39" spans="1:26" ht="15.75" customHeight="1">
       <c r="A39" s="37"/>
-      <c r="B39" s="133"/>
-      <c r="C39" s="113"/>
-      <c r="D39" s="113"/>
-      <c r="E39" s="113"/>
-      <c r="F39" s="113"/>
-      <c r="G39" s="113"/>
-      <c r="H39" s="113"/>
+      <c r="B39" s="104"/>
+      <c r="C39" s="114"/>
+      <c r="D39" s="114"/>
+      <c r="E39" s="114"/>
+      <c r="F39" s="114"/>
+      <c r="G39" s="114"/>
+      <c r="H39" s="114"/>
       <c r="I39" s="57"/>
       <c r="J39" s="58"/>
       <c r="K39" s="57"/>
@@ -3112,25 +3108,25 @@
     <row r="40" spans="1:26" ht="4.5" customHeight="1">
       <c r="A40" s="1"/>
       <c r="B40" s="61"/>
-      <c r="C40" s="134"/>
-      <c r="D40" s="135"/>
-      <c r="E40" s="135"/>
-      <c r="F40" s="135"/>
-      <c r="G40" s="135"/>
-      <c r="H40" s="135"/>
-      <c r="I40" s="135"/>
-      <c r="J40" s="135"/>
-      <c r="K40" s="135"/>
-      <c r="L40" s="135"/>
-      <c r="M40" s="135"/>
-      <c r="N40" s="135"/>
-      <c r="O40" s="135"/>
-      <c r="P40" s="135"/>
-      <c r="Q40" s="135"/>
-      <c r="R40" s="135"/>
-      <c r="S40" s="135"/>
-      <c r="T40" s="135"/>
-      <c r="U40" s="108"/>
+      <c r="C40" s="105"/>
+      <c r="D40" s="138"/>
+      <c r="E40" s="138"/>
+      <c r="F40" s="138"/>
+      <c r="G40" s="138"/>
+      <c r="H40" s="138"/>
+      <c r="I40" s="138"/>
+      <c r="J40" s="138"/>
+      <c r="K40" s="138"/>
+      <c r="L40" s="138"/>
+      <c r="M40" s="138"/>
+      <c r="N40" s="138"/>
+      <c r="O40" s="138"/>
+      <c r="P40" s="138"/>
+      <c r="Q40" s="138"/>
+      <c r="R40" s="138"/>
+      <c r="S40" s="138"/>
+      <c r="T40" s="138"/>
+      <c r="U40" s="137"/>
       <c r="V40" s="1"/>
       <c r="W40" s="1"/>
       <c r="X40" s="1"/>
@@ -3139,32 +3135,32 @@
     </row>
     <row r="41" spans="1:26" ht="30" customHeight="1">
       <c r="A41" s="62"/>
-      <c r="B41" s="136" t="s">
+      <c r="B41" s="106" t="s">
         <v>56</v>
       </c>
-      <c r="C41" s="91"/>
-      <c r="D41" s="91"/>
-      <c r="E41" s="91"/>
-      <c r="F41" s="91"/>
-      <c r="G41" s="91"/>
-      <c r="H41" s="91"/>
-      <c r="I41" s="91"/>
-      <c r="J41" s="137" t="s">
+      <c r="C41" s="111"/>
+      <c r="D41" s="111"/>
+      <c r="E41" s="111"/>
+      <c r="F41" s="111"/>
+      <c r="G41" s="111"/>
+      <c r="H41" s="111"/>
+      <c r="I41" s="111"/>
+      <c r="J41" s="107" t="s">
         <v>57</v>
       </c>
-      <c r="K41" s="91"/>
-      <c r="L41" s="91"/>
-      <c r="M41" s="91"/>
-      <c r="N41" s="91"/>
-      <c r="O41" s="106"/>
-      <c r="P41" s="138" t="s">
+      <c r="K41" s="111"/>
+      <c r="L41" s="111"/>
+      <c r="M41" s="111"/>
+      <c r="N41" s="111"/>
+      <c r="O41" s="112"/>
+      <c r="P41" s="108" t="s">
         <v>58</v>
       </c>
-      <c r="Q41" s="91"/>
-      <c r="R41" s="91"/>
-      <c r="S41" s="91"/>
-      <c r="T41" s="91"/>
-      <c r="U41" s="106"/>
+      <c r="Q41" s="111"/>
+      <c r="R41" s="111"/>
+      <c r="S41" s="111"/>
+      <c r="T41" s="111"/>
+      <c r="U41" s="112"/>
       <c r="V41" s="62"/>
       <c r="W41" s="62"/>
       <c r="X41" s="62"/>
@@ -3173,26 +3169,26 @@
     </row>
     <row r="42" spans="1:26" ht="30" customHeight="1">
       <c r="A42" s="62"/>
-      <c r="B42" s="129"/>
-      <c r="C42" s="107"/>
-      <c r="D42" s="107"/>
-      <c r="E42" s="107"/>
-      <c r="F42" s="107"/>
-      <c r="G42" s="107"/>
-      <c r="H42" s="107"/>
-      <c r="I42" s="107"/>
-      <c r="J42" s="132"/>
-      <c r="K42" s="107"/>
-      <c r="L42" s="107"/>
-      <c r="M42" s="107"/>
-      <c r="N42" s="107"/>
-      <c r="O42" s="108"/>
-      <c r="P42" s="139"/>
-      <c r="Q42" s="107"/>
-      <c r="R42" s="107"/>
-      <c r="S42" s="107"/>
-      <c r="T42" s="107"/>
-      <c r="U42" s="108"/>
+      <c r="B42" s="101"/>
+      <c r="C42" s="136"/>
+      <c r="D42" s="136"/>
+      <c r="E42" s="136"/>
+      <c r="F42" s="136"/>
+      <c r="G42" s="136"/>
+      <c r="H42" s="136"/>
+      <c r="I42" s="136"/>
+      <c r="J42" s="135"/>
+      <c r="K42" s="136"/>
+      <c r="L42" s="136"/>
+      <c r="M42" s="136"/>
+      <c r="N42" s="136"/>
+      <c r="O42" s="137"/>
+      <c r="P42" s="109"/>
+      <c r="Q42" s="136"/>
+      <c r="R42" s="136"/>
+      <c r="S42" s="136"/>
+      <c r="T42" s="136"/>
+      <c r="U42" s="137"/>
       <c r="V42" s="62"/>
       <c r="W42" s="62"/>
       <c r="X42" s="62"/>
@@ -3201,30 +3197,30 @@
     </row>
     <row r="43" spans="1:26" ht="30" customHeight="1">
       <c r="A43" s="62"/>
-      <c r="B43" s="130" t="s">
+      <c r="B43" s="102" t="s">
         <v>59</v>
       </c>
-      <c r="C43" s="113"/>
-      <c r="D43" s="113"/>
-      <c r="E43" s="113"/>
-      <c r="F43" s="113"/>
-      <c r="G43" s="113"/>
-      <c r="H43" s="113"/>
-      <c r="I43" s="113"/>
-      <c r="J43" s="124"/>
-      <c r="K43" s="113"/>
-      <c r="L43" s="113"/>
-      <c r="M43" s="113"/>
-      <c r="N43" s="113"/>
-      <c r="O43" s="114"/>
-      <c r="P43" s="140" t="s">
+      <c r="C43" s="114"/>
+      <c r="D43" s="114"/>
+      <c r="E43" s="114"/>
+      <c r="F43" s="114"/>
+      <c r="G43" s="114"/>
+      <c r="H43" s="114"/>
+      <c r="I43" s="114"/>
+      <c r="J43" s="113"/>
+      <c r="K43" s="114"/>
+      <c r="L43" s="114"/>
+      <c r="M43" s="114"/>
+      <c r="N43" s="114"/>
+      <c r="O43" s="115"/>
+      <c r="P43" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="Q43" s="113"/>
-      <c r="R43" s="113"/>
-      <c r="S43" s="113"/>
-      <c r="T43" s="113"/>
-      <c r="U43" s="114"/>
+      <c r="Q43" s="114"/>
+      <c r="R43" s="114"/>
+      <c r="S43" s="114"/>
+      <c r="T43" s="114"/>
+      <c r="U43" s="115"/>
       <c r="V43" s="62"/>
       <c r="W43" s="62"/>
       <c r="X43" s="62"/>

</xml_diff>